<commit_message>
corrected text color in completed consultancy and text in students alumini tab
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB55A4FD-B23B-4777-ABF4-BA39899C68C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB9B819-57FE-468B-A5CC-FE9B6D8B7DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CoreFaculty" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="92">
   <si>
     <t>Name</t>
   </si>
@@ -271,6 +271,39 @@
   </si>
   <si>
     <t>Pedestrian Cross Flow Modelling, Non-Motorized Safety, Traffic Safety, Driver Behaviour, Traffic flow modeling • Transportation Environment • Travel behavior, Sustainable Transportation • Freight Transportation</t>
+  </si>
+  <si>
+    <t>Prof. Venkaiah Chowdary</t>
+  </si>
+  <si>
+    <t>Professor</t>
+  </si>
+  <si>
+    <t>vc@nitw.ac.in</t>
+  </si>
+  <si>
+    <t>Characterization for asphalt binders and mixtures; asphalt pavement analysis, design and evaluation; quantification of roadway and railway traffic noise.</t>
+  </si>
+  <si>
+    <t>https://erp.nitw.ac.in/ext/profile/getUserImage/ce-vc</t>
+  </si>
+  <si>
+    <t>https://erp.nitw.ac.in/ext/profile/ce-vc</t>
+  </si>
+  <si>
+    <t>Prof. S. Shankar</t>
+  </si>
+  <si>
+    <t>ss@nitw.ac.in</t>
+  </si>
+  <si>
+    <t>Low Volume Roads, Pavement Analysis and Design, Pavement Management System, Pavement Material characterization, Geo-Synthetic Applications in Pavements and Marginal and Innovative Materials in LVRs</t>
+  </si>
+  <si>
+    <t>https://erp.nitw.ac.in/ext/profile/getUserImage/ce-ss</t>
+  </si>
+  <si>
+    <t>https://erp.nitw.ac.in/ext/profile/ce-ss</t>
   </si>
 </sst>
 </file>
@@ -606,7 +639,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
@@ -735,36 +768,86 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6">
+        <v>9849102935</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7">
+        <v>8332969252</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>24</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D8" t="s">
         <v>25</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E8" t="s">
         <v>26</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F8" t="s">
         <v>28</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G8" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G6">
-    <sortCondition ref="A2:A6"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G8">
+    <sortCondition ref="A5:A8"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{E5822289-CFEA-422D-AC65-BCF8A3E05343}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{F776B85C-FD73-46BF-85F1-C6C749158FA3}"/>
     <hyperlink ref="F3" r:id="rId3" xr:uid="{51DD2074-866B-453C-9084-5D9B38722E68}"/>
     <hyperlink ref="D5" r:id="rId4" xr:uid="{EDD927B0-11EA-4F61-B44F-01306BE1BCF1}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{AF349A3B-65A6-4BED-A302-FEA82F060327}"/>
+    <hyperlink ref="F7" r:id="rId6" xr:uid="{EE795596-A6E6-4391-AB06-1414421C11AD}"/>
+    <hyperlink ref="D6" r:id="rId7" display="mailto:ss@nitw.ac.in" xr:uid="{3D758237-1E6D-4D2D-8FDA-8431CAFEB283}"/>
+    <hyperlink ref="F6" r:id="rId8" xr:uid="{3EDEE717-2E36-473B-8A47-61F2C9ED6B20}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
guest faculty mock data update
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB9B819-57FE-468B-A5CC-FE9B6D8B7DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BB82E1-A9B5-4A7F-B0B4-E1C6030D35B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CoreFaculty" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="144">
   <si>
     <t>Name</t>
   </si>
@@ -304,13 +304,169 @@
   </si>
   <si>
     <t>https://erp.nitw.ac.in/ext/profile/ce-ss</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Research Areas</t>
+  </si>
+  <si>
+    <t>faculty1.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Ananya Sharma</t>
+  </si>
+  <si>
+    <t>+91 98765 43210</t>
+  </si>
+  <si>
+    <t>ananya.sharma@university.edu</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence, Machine Learning, Data Analytics</t>
+  </si>
+  <si>
+    <t>faculty2.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Rahul Verma</t>
+  </si>
+  <si>
+    <t>+91 98765 43211</t>
+  </si>
+  <si>
+    <t>rahul.verma@university.edu</t>
+  </si>
+  <si>
+    <t>Computer Vision, Image Processing, Deep Learning</t>
+  </si>
+  <si>
+    <t>faculty3.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Priya Nair</t>
+  </si>
+  <si>
+    <t>+91 98765 43212</t>
+  </si>
+  <si>
+    <t>priya.nair@university.edu</t>
+  </si>
+  <si>
+    <t>Cyber Security, Network Security, Cryptography</t>
+  </si>
+  <si>
+    <t>faculty4.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Karthik Reddy</t>
+  </si>
+  <si>
+    <t>+91 98765 43213</t>
+  </si>
+  <si>
+    <t>karthik.reddy@university.edu</t>
+  </si>
+  <si>
+    <t>Internet of Things (IoT), Embedded Systems</t>
+  </si>
+  <si>
+    <t>faculty5.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Sneha Gupta</t>
+  </si>
+  <si>
+    <t>+91 98765 43214</t>
+  </si>
+  <si>
+    <t>sneha.gupta@university.edu</t>
+  </si>
+  <si>
+    <t>Natural Language Processing, Generative AI</t>
+  </si>
+  <si>
+    <t>faculty6.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Arjun Mehta</t>
+  </si>
+  <si>
+    <t>+91 98765 43215</t>
+  </si>
+  <si>
+    <t>arjun.mehta@university.edu</t>
+  </si>
+  <si>
+    <t>Big Data Analytics, Cloud Computing</t>
+  </si>
+  <si>
+    <t>faculty7.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Neha Kapoor</t>
+  </si>
+  <si>
+    <t>+91 98765 43216</t>
+  </si>
+  <si>
+    <t>neha.kapoor@university.edu</t>
+  </si>
+  <si>
+    <t>Human-Computer Interaction, UX Design</t>
+  </si>
+  <si>
+    <t>faculty8.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Vikram Singh</t>
+  </si>
+  <si>
+    <t>+91 98765 43217</t>
+  </si>
+  <si>
+    <t>vikram.singh@university.edu</t>
+  </si>
+  <si>
+    <t>Robotics, Autonomous Systems</t>
+  </si>
+  <si>
+    <t>faculty9.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Pooja Menon</t>
+  </si>
+  <si>
+    <t>+91 98765 43218</t>
+  </si>
+  <si>
+    <t>pooja.menon@university.edu</t>
+  </si>
+  <si>
+    <t>Data Science, Business Intelligence</t>
+  </si>
+  <si>
+    <t>faculty10.jpg</t>
+  </si>
+  <si>
+    <t>Dr. Rohan Das</t>
+  </si>
+  <si>
+    <t>+91 98765 43219</t>
+  </si>
+  <si>
+    <t>rohan.das@university.edu</t>
+  </si>
+  <si>
+    <t>Software Engineering, Distributed Systems</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,6 +487,14 @@
       <color rgb="FF212529"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -354,10 +518,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -944,12 +1114,236 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06D969DC-6FC0-4E4D-B105-6F6F4232277C}">
-  <dimension ref="D3:F3"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+    <col min="4" max="4" width="37.85546875" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="4:6" x14ac:dyDescent="0.25">
-      <c r="D3" s="2"/>
-      <c r="F3" s="2"/>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>139</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated faculty designation, social media animation
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34BB82E1-A9B5-4A7F-B0B4-E1C6030D35B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EE9337-1F16-47D7-AF33-F9D193924AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CoreFaculty" sheetId="1" r:id="rId1"/>
@@ -872,7 +872,7 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>8879425755</v>
@@ -918,7 +918,7 @@
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="C5">
         <v>8332969262</v>
@@ -941,7 +941,7 @@
         <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>82</v>
       </c>
       <c r="C6">
         <v>9849102935</v>

</xml_diff>

<commit_message>
active blue button and contact us tab
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA08F108-13DC-486E-8FF0-05E21A9A6674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7855879-5D8C-42F9-A939-52E9C584BF33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="145">
   <si>
     <t>Name</t>
   </si>
@@ -313,9 +313,6 @@
     <t>Research Areas</t>
   </si>
   <si>
-    <t>faculty1.jpg</t>
-  </si>
-  <si>
     <t>Dr. Ananya Sharma</t>
   </si>
   <si>
@@ -328,9 +325,6 @@
     <t>Artificial Intelligence, Machine Learning, Data Analytics</t>
   </si>
   <si>
-    <t>faculty2.jpg</t>
-  </si>
-  <si>
     <t>Dr. Rahul Verma</t>
   </si>
   <si>
@@ -343,9 +337,6 @@
     <t>Computer Vision, Image Processing, Deep Learning</t>
   </si>
   <si>
-    <t>faculty3.jpg</t>
-  </si>
-  <si>
     <t>Dr. Priya Nair</t>
   </si>
   <si>
@@ -358,9 +349,6 @@
     <t>Cyber Security, Network Security, Cryptography</t>
   </si>
   <si>
-    <t>faculty4.jpg</t>
-  </si>
-  <si>
     <t>Dr. Karthik Reddy</t>
   </si>
   <si>
@@ -373,9 +361,6 @@
     <t>Internet of Things (IoT), Embedded Systems</t>
   </si>
   <si>
-    <t>faculty5.jpg</t>
-  </si>
-  <si>
     <t>Dr. Sneha Gupta</t>
   </si>
   <si>
@@ -388,9 +373,6 @@
     <t>Natural Language Processing, Generative AI</t>
   </si>
   <si>
-    <t>faculty6.jpg</t>
-  </si>
-  <si>
     <t>Dr. Arjun Mehta</t>
   </si>
   <si>
@@ -403,9 +385,6 @@
     <t>Big Data Analytics, Cloud Computing</t>
   </si>
   <si>
-    <t>faculty7.jpg</t>
-  </si>
-  <si>
     <t>Dr. Neha Kapoor</t>
   </si>
   <si>
@@ -418,9 +397,6 @@
     <t>Human-Computer Interaction, UX Design</t>
   </si>
   <si>
-    <t>faculty8.jpg</t>
-  </si>
-  <si>
     <t>Dr. Vikram Singh</t>
   </si>
   <si>
@@ -433,9 +409,6 @@
     <t>Robotics, Autonomous Systems</t>
   </si>
   <si>
-    <t>faculty9.jpg</t>
-  </si>
-  <si>
     <t>Dr. Pooja Menon</t>
   </si>
   <si>
@@ -446,9 +419,6 @@
   </si>
   <si>
     <t>Data Science, Business Intelligence</t>
-  </si>
-  <si>
-    <t>faculty10.jpg</t>
   </si>
   <si>
     <t>Dr. Rohan Das</t>
@@ -1261,203 +1231,183 @@
     </row>
     <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>99</v>
-      </c>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>104</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="F5" s="4" t="s">
         <v>109</v>
       </c>
+      <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>114</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>119</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>124</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>31</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>129</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>134</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>139</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="F11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1503,9 +1453,7 @@
       <c r="D2">
         <v>1970</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="E2" s="4"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -1520,9 +1468,7 @@
       <c r="D3">
         <v>1973</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>99</v>
-      </c>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -1537,9 +1483,7 @@
       <c r="D4">
         <v>1978</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>104</v>
-      </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -1554,9 +1498,7 @@
       <c r="D5">
         <v>1970</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>109</v>
-      </c>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -1571,9 +1513,7 @@
       <c r="D6">
         <v>1973</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>114</v>
-      </c>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1588,9 +1528,7 @@
       <c r="D7">
         <v>1978</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1605,9 +1543,7 @@
       <c r="D8">
         <v>1997</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>124</v>
-      </c>
+      <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1622,9 +1558,7 @@
       <c r="D9">
         <v>1970</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>129</v>
-      </c>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1639,9 +1573,7 @@
       <c r="D10">
         <v>1971</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>134</v>
-      </c>
+      <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1656,9 +1588,7 @@
       <c r="D11">
         <v>1972</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1673,9 +1603,7 @@
       <c r="D12">
         <v>1973</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -1690,9 +1618,7 @@
       <c r="D13">
         <v>1972</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -1707,9 +1633,7 @@
       <c r="D14">
         <v>1980</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -1724,9 +1648,7 @@
       <c r="D15">
         <v>2007</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -1741,9 +1663,7 @@
       <c r="D16">
         <v>1981</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
@@ -1758,9 +1678,7 @@
       <c r="D17">
         <v>1975</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
@@ -1775,9 +1693,7 @@
       <c r="D18">
         <v>1981</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
@@ -1792,9 +1708,7 @@
       <c r="D19">
         <v>2007</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E19" s="4"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -1809,9 +1723,7 @@
       <c r="D20">
         <v>1991</v>
       </c>
-      <c r="E20" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E20" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
@@ -1826,9 +1738,7 @@
       <c r="D21">
         <v>1993</v>
       </c>
-      <c r="E21" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
@@ -1843,9 +1753,7 @@
       <c r="D22">
         <v>1993</v>
       </c>
-      <c r="E22" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
@@ -1860,9 +1768,7 @@
       <c r="D23">
         <v>2003</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E23" s="4"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
@@ -1877,9 +1783,7 @@
       <c r="D24">
         <v>2003</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E24" s="4"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
@@ -1894,9 +1798,7 @@
       <c r="D25">
         <v>2004</v>
       </c>
-      <c r="E25" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E25" s="4"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26">
@@ -1911,9 +1813,7 @@
       <c r="D26">
         <v>2003</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E26" s="4"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27">
@@ -1928,9 +1828,7 @@
       <c r="D27">
         <v>2004</v>
       </c>
-      <c r="E27" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E27" s="4"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28">
@@ -1945,9 +1843,7 @@
       <c r="D28">
         <v>2005</v>
       </c>
-      <c r="E28" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E28" s="4"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29">
@@ -1962,9 +1858,7 @@
       <c r="D29">
         <v>2005</v>
       </c>
-      <c r="E29" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E29" s="4"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30">
@@ -1979,9 +1873,7 @@
       <c r="D30">
         <v>2013</v>
       </c>
-      <c r="E30" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31">
@@ -1996,9 +1888,7 @@
       <c r="D31">
         <v>2017</v>
       </c>
-      <c r="E31" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E31" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2019,7 +1909,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>0</v>
@@ -2039,7 +1929,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="C2" s="9">
         <v>1968</v>
@@ -2047,16 +1937,14 @@
       <c r="D2" s="9">
         <v>1970</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="E2" s="4"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="C3" s="9">
         <v>1970</v>
@@ -2064,16 +1952,14 @@
       <c r="D3" s="9">
         <v>1978</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>99</v>
-      </c>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C4" s="9">
         <v>1978</v>
@@ -2081,16 +1967,14 @@
       <c r="D4" s="9">
         <v>1987</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>104</v>
-      </c>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C5" s="9">
         <v>1987</v>
@@ -2098,16 +1982,14 @@
       <c r="D5" s="9">
         <v>1990</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>109</v>
-      </c>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="C6" s="9">
         <v>1990</v>
@@ -2115,16 +1997,14 @@
       <c r="D6" s="9">
         <v>1993</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>114</v>
-      </c>
+      <c r="E6" s="4"/>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C7" s="9">
         <v>1993</v>
@@ -2132,16 +2012,14 @@
       <c r="D7" s="9">
         <v>1996</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="C8" s="9">
         <v>1996</v>
@@ -2149,16 +2027,14 @@
       <c r="D8" s="9">
         <v>1999</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>124</v>
-      </c>
+      <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7">
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C9" s="9">
         <v>1999</v>
@@ -2166,16 +2042,14 @@
       <c r="D9" s="9">
         <v>2002</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>129</v>
-      </c>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7">
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C10" s="9">
         <v>2002</v>
@@ -2183,16 +2057,14 @@
       <c r="D10" s="9">
         <v>2005</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>134</v>
-      </c>
+      <c r="E10" s="4"/>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7">
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C11" s="9">
         <v>2005</v>
@@ -2200,16 +2072,14 @@
       <c r="D11" s="9">
         <v>2006</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7">
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C12" s="9">
         <v>2006</v>
@@ -2217,16 +2087,14 @@
       <c r="D12" s="9">
         <v>2018</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7">
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="C13" s="9">
         <v>2018</v>
@@ -2234,16 +2102,14 @@
       <c r="D13" s="9">
         <v>2022</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E13" s="4"/>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7">
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C14" s="9">
         <v>2022</v>
@@ -2251,26 +2117,22 @@
       <c r="D14" s="9">
         <v>2024</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>139</v>
-      </c>
+      <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7">
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C15" s="9">
         <v>2024</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>139</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E16" s="4"/>

</xml_diff>

<commit_message>
previous faculty photos update
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9328B2-0F97-4958-83F5-DCCFDDBA18C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="CoreFaculty" sheetId="1" r:id="rId1"/>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="158">
   <si>
     <t>Name</t>
   </si>
@@ -494,12 +493,21 @@
   </si>
   <si>
     <t>images/Previous Faculty/N. Sadguna.jpg</t>
+  </si>
+  <si>
+    <t>images/Previous Faculty/K. Appala Raju.jpg</t>
+  </si>
+  <si>
+    <t>images/Previous Faculty/Dr. Francis Christopher.jpg</t>
+  </si>
+  <si>
+    <t>images/Previous Faculty/P. Sasanka Bhushan.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -949,7 +957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1144,18 +1152,18 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G8">
+  <sortState ref="A2:G8">
     <sortCondition ref="A5:A8"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="D4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="D6" r:id="rId7" display="mailto:ss@nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F6" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D4" r:id="rId1"/>
+    <hyperlink ref="D3" r:id="rId2"/>
+    <hyperlink ref="F3" r:id="rId3"/>
+    <hyperlink ref="D5" r:id="rId4"/>
+    <hyperlink ref="D7" r:id="rId5"/>
+    <hyperlink ref="F7" r:id="rId6"/>
+    <hyperlink ref="D6" r:id="rId7" display="mailto:ss@nitw.ac.in"/>
+    <hyperlink ref="F6" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId9"/>
@@ -1163,7 +1171,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1243,18 +1251,18 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E4">
+  <sortState ref="A2:E4">
     <sortCondition ref="A2:A4"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="E3" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1472,7 +1480,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1758,7 +1766,9 @@
       <c r="D18">
         <v>2000</v>
       </c>
-      <c r="E18" s="4"/>
+      <c r="E18" s="4" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
@@ -1773,7 +1783,9 @@
       <c r="D19">
         <v>1993</v>
       </c>
-      <c r="E19" s="4"/>
+      <c r="E19" s="4" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
@@ -1949,7 +1961,9 @@
       <c r="D30">
         <v>2017</v>
       </c>
-      <c r="E30" s="4"/>
+      <c r="E30" s="4" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E31" s="4"/>
@@ -1960,7 +1974,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2286,9 +2300,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E15" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
-    <hyperlink ref="E13" r:id="rId2" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
-    <hyperlink ref="E10" r:id="rId3" xr:uid="{CF961E56-8C58-43C7-9E8E-C4C1CF4ECF88}"/>
+    <hyperlink ref="E15" r:id="rId1"/>
+    <hyperlink ref="E13" r:id="rId2"/>
+    <hyperlink ref="E10" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId4"/>

</xml_diff>

<commit_message>
core faculty css and IDs update
</commit_message>
<xml_diff>
--- a/excels/faculty.xlsx
+++ b/excels/faculty.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF1586BB-83AC-43AF-A2D9-B22E9CE76B11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD31B2D8-A205-41C2-B8F9-1F9CB3A2C4D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="183">
   <si>
     <t>Name</t>
   </si>
@@ -521,13 +521,70 @@
   </si>
   <si>
     <t>PATENTS</t>
+  </si>
+  <si>
+    <t>PhD Institute</t>
+  </si>
+  <si>
+    <t>Masters Institute</t>
+  </si>
+  <si>
+    <t>Indian Institute of Technology Roorkee</t>
+  </si>
+  <si>
+    <t>Indian Institute of Technology Guwahati</t>
+  </si>
+  <si>
+    <t>IIT Bombay</t>
+  </si>
+  <si>
+    <t>NIT Warangal</t>
+  </si>
+  <si>
+    <t>JNTU Hyderabad</t>
+  </si>
+  <si>
+    <t>National Institute of Technology Warangal</t>
+  </si>
+  <si>
+    <t>Indian Institute of Technology Madras</t>
+  </si>
+  <si>
+    <t>IIT Kharagpur</t>
+  </si>
+  <si>
+    <t>ORCID</t>
+  </si>
+  <si>
+    <t>Scopus</t>
+  </si>
+  <si>
+    <t>GoogleScholar</t>
+  </si>
+  <si>
+    <t>0000-0002-1680-2089</t>
+  </si>
+  <si>
+    <t>0000-0002-0636-1355</t>
+  </si>
+  <si>
+    <t>0000-0001-6648-2493</t>
+  </si>
+  <si>
+    <t>0000-0002-5458-3972</t>
+  </si>
+  <si>
+    <t>0000-0001-6156-4625</t>
+  </si>
+  <si>
+    <t>0000-0001-9721-1557</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -570,16 +627,28 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF212529"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -659,12 +728,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDEE2E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDEE2E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDEE2E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDEE2E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -696,6 +780,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -977,23 +1068,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="21.42578125" customWidth="1"/>
     <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="17.5703125" customWidth="1"/>
-    <col min="7" max="7" width="21.42578125" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="80.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="38.42578125" customWidth="1"/>
-    <col min="13" max="13" width="7.140625" customWidth="1"/>
-    <col min="14" max="15" width="9" customWidth="1"/>
+    <col min="7" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="43" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="21.42578125" customWidth="1"/>
+    <col min="13" max="13" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="80.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="38.42578125" customWidth="1"/>
+    <col min="18" max="18" width="7.140625" customWidth="1"/>
+    <col min="19" max="20" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1016,25 +1110,40 @@
         <v>159</v>
       </c>
       <c r="H1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I1" t="s">
+        <v>165</v>
+      </c>
+      <c r="J1" t="s">
+        <v>174</v>
+      </c>
+      <c r="K1" t="s">
+        <v>175</v>
+      </c>
+      <c r="L1" t="s">
+        <v>176</v>
+      </c>
+      <c r="M1" t="s">
         <v>1</v>
       </c>
-      <c r="I1" t="s">
+      <c r="N1" t="s">
         <v>2</v>
       </c>
-      <c r="J1" t="s">
+      <c r="O1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" t="s">
+      <c r="P1" t="s">
         <v>4</v>
       </c>
-      <c r="L1" t="s">
+      <c r="Q1" t="s">
         <v>20</v>
       </c>
-      <c r="M1" t="s">
+      <c r="R1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -1044,26 +1153,38 @@
       <c r="D2">
         <v>8</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="K2">
+        <v>55978788300</v>
+      </c>
+      <c r="M2" t="s">
         <v>31</v>
       </c>
-      <c r="I2">
+      <c r="N2">
         <v>8332969421</v>
       </c>
-      <c r="J2" t="s">
+      <c r="O2" t="s">
         <v>32</v>
       </c>
-      <c r="K2" t="s">
+      <c r="P2" t="s">
         <v>33</v>
       </c>
-      <c r="L2" t="s">
+      <c r="Q2" t="s">
         <v>34</v>
       </c>
-      <c r="M2" t="s">
+      <c r="R2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1079,26 +1200,38 @@
       <c r="F3">
         <v>1</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="J3" t="s">
+        <v>178</v>
+      </c>
+      <c r="K3">
+        <v>56237024300</v>
+      </c>
+      <c r="M3" t="s">
         <v>31</v>
       </c>
-      <c r="I3">
+      <c r="N3">
         <v>8879425755</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="O3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K3" t="s">
+      <c r="P3" t="s">
         <v>78</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="Q3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="M3" t="s">
+      <c r="R3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -1111,26 +1244,38 @@
       <c r="E4">
         <v>8</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="I4" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="J4" t="s">
+        <v>179</v>
+      </c>
+      <c r="K4">
+        <v>55024478300</v>
+      </c>
+      <c r="M4" t="s">
         <v>6</v>
       </c>
-      <c r="I4" t="s">
+      <c r="N4" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L4" t="s">
+      <c r="Q4" t="s">
         <v>10</v>
       </c>
-      <c r="M4" t="s">
+      <c r="R4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1146,26 +1291,38 @@
       <c r="F5">
         <v>1</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="J5" t="s">
+        <v>180</v>
+      </c>
+      <c r="K5">
+        <v>57193253075</v>
+      </c>
+      <c r="M5" t="s">
         <v>80</v>
       </c>
-      <c r="I5">
+      <c r="N5">
         <v>8332969262</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="O5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K5" t="s">
+      <c r="P5" t="s">
         <v>38</v>
       </c>
-      <c r="L5" t="s">
+      <c r="Q5" t="s">
         <v>39</v>
       </c>
-      <c r="M5" t="s">
+      <c r="R5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1181,26 +1338,38 @@
       <c r="F6">
         <v>3</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="J6" t="s">
+        <v>181</v>
+      </c>
+      <c r="K6">
+        <v>57211683260</v>
+      </c>
+      <c r="M6" t="s">
         <v>80</v>
       </c>
-      <c r="I6">
+      <c r="N6">
         <v>9849102935</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="O6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="K6" t="s">
+      <c r="P6" t="s">
         <v>87</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="Q6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="M6" t="s">
+      <c r="R6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>79</v>
       </c>
@@ -1213,26 +1382,32 @@
       <c r="E7">
         <v>7</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="M7" t="s">
         <v>80</v>
       </c>
-      <c r="I7">
+      <c r="N7">
         <v>8332969252</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="O7" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K7" t="s">
+      <c r="P7" t="s">
         <v>82</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="Q7" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="M7" t="s">
+      <c r="R7" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -1245,35 +1420,47 @@
       <c r="E8">
         <v>9</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="J8" t="s">
+        <v>182</v>
+      </c>
+      <c r="K8">
+        <v>57192237169</v>
+      </c>
+      <c r="M8" t="s">
         <v>12</v>
       </c>
-      <c r="J8" t="s">
+      <c r="O8" t="s">
         <v>25</v>
       </c>
-      <c r="K8" t="s">
+      <c r="P8" t="s">
         <v>26</v>
       </c>
-      <c r="L8" t="s">
+      <c r="Q8" t="s">
         <v>28</v>
       </c>
-      <c r="M8" t="s">
+      <c r="R8" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R8">
     <sortCondition ref="A5:A8"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="J4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="J3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="L3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="J5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="J7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="L7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="J6" r:id="rId7" display="mailto:ss@nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="L6" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="O4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="O3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="Q3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="O5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="O7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="Q7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="O6" r:id="rId7" display="mailto:ss@nitw.ac.in" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="Q6" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId9"/>

</xml_diff>